<commit_message>
!SECURITY UPDATE: update security
Added php checks to all files that needed it
</commit_message>
<xml_diff>
--- a/config/tiktokDummEntry1.xlsx
+++ b/config/tiktokDummEntry1.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinantolihao/ApacheProjects/ITPROG/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1395F551-01EA-7248-954E-7EB26BC52A51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3FA230D-8E75-964C-B6C6-898110846252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5980" yWindow="4420" windowWidth="27240" windowHeight="16440" xr2:uid="{EAD12DD5-832B-D740-A33E-2D7642D34CB4}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" xr2:uid="{EAD12DD5-832B-D740-A33E-2D7642D34CB4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="tiktok_shop_dummy_orders" localSheetId="0">Sheet1!$A$1:$W$11</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -35,8 +38,42 @@
 </workbook>
 </file>
 
+<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
+  <connection id="1" xr16:uid="{12E85BF4-1DBF-7446-A7B3-002A922292FD}" name="tiktok_shop_dummy_orders" type="6" refreshedVersion="8" background="1" saveData="1">
+    <textPr codePage="10000" sourceFile="/Users/martinantolihao/Downloads/tiktok_shop_dummy_orders.csv" tab="0" comma="1">
+      <textFields count="23">
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+        <textField/>
+      </textFields>
+    </textPr>
+  </connection>
+</connections>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="50">
   <si>
     <t>Order ID</t>
   </si>
@@ -107,29 +144,104 @@
     <t>Purchase Channel</t>
   </si>
   <si>
-    <t>x</t>
-  </si>
-  <si>
-    <t>TK-0009812</t>
-  </si>
-  <si>
-    <t>TK-0001</t>
-  </si>
-  <si>
-    <t>TK-0008</t>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>TT-H001-03</t>
+  </si>
+  <si>
+    <t>FBL</t>
+  </si>
+  <si>
+    <t>WH-A1</t>
+  </si>
+  <si>
+    <t>TRK8839101</t>
+  </si>
+  <si>
+    <t>Standard</t>
+  </si>
+  <si>
+    <t>COD</t>
+  </si>
+  <si>
+    <t>PKG-5001</t>
+  </si>
+  <si>
+    <t>TikTok Shop</t>
+  </si>
+  <si>
+    <t>TT-S001-03</t>
+  </si>
+  <si>
+    <t>TT-H002-03</t>
+  </si>
+  <si>
+    <t>TT-H003-03</t>
+  </si>
+  <si>
+    <t>WH-B2</t>
+  </si>
+  <si>
+    <t>TRK7721190</t>
+  </si>
+  <si>
+    <t>Express</t>
+  </si>
+  <si>
+    <t>Card</t>
+  </si>
+  <si>
+    <t>PKG-5002</t>
+  </si>
+  <si>
+    <t>TT-S002-03</t>
+  </si>
+  <si>
+    <t>WH-C3</t>
+  </si>
+  <si>
+    <t>TRK6651029</t>
+  </si>
+  <si>
+    <t>E-Wallet</t>
+  </si>
+  <si>
+    <t>PKG-5003</t>
+  </si>
+  <si>
+    <t>order placed</t>
+  </si>
+  <si>
+    <t>TT_1001</t>
+  </si>
+  <si>
+    <t>TT_1002</t>
+  </si>
+  <si>
+    <t>TT_1003</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -152,8 +264,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -169,6 +282,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="tiktok_shop_dummy_orders" connectionId="1" xr16:uid="{2C92BE3D-C654-E647-B2AD-8770167E18B9}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -488,8 +605,33 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F1BB48F-0F3C-C54F-899E-B2C995AC77C7}">
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="24.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="15.83203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -564,147 +706,716 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" t="s">
         <v>25</v>
       </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" t="s">
-        <v>23</v>
-      </c>
-      <c r="N2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O2" t="s">
-        <v>23</v>
-      </c>
-      <c r="P2" t="s">
-        <v>23</v>
+      <c r="F2">
+        <v>700</v>
+      </c>
+      <c r="G2">
+        <v>799</v>
+      </c>
+      <c r="H2">
+        <v>80</v>
+      </c>
+      <c r="I2">
+        <v>50</v>
+      </c>
+      <c r="J2">
+        <v>669</v>
+      </c>
+      <c r="K2">
+        <v>80</v>
+      </c>
+      <c r="L2">
+        <v>120</v>
+      </c>
+      <c r="M2">
+        <v>20</v>
+      </c>
+      <c r="N2">
+        <v>20</v>
+      </c>
+      <c r="O2">
+        <v>749</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
       </c>
       <c r="Q2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="R2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="S2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="T2" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="U2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="V2" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="W2" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
         <v>23</v>
       </c>
       <c r="C3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" s="1">
+        <v>850</v>
+      </c>
+      <c r="G3">
+        <v>699</v>
+      </c>
+      <c r="H3">
+        <v>70</v>
+      </c>
+      <c r="I3">
+        <v>40</v>
+      </c>
+      <c r="J3">
+        <v>589</v>
+      </c>
+      <c r="K3">
+        <v>60</v>
+      </c>
+      <c r="L3">
+        <v>100</v>
+      </c>
+      <c r="M3">
+        <v>20</v>
+      </c>
+      <c r="N3">
+        <v>20</v>
+      </c>
+      <c r="O3">
+        <v>749</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>26</v>
+      </c>
+      <c r="R3" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3" t="s">
+        <v>28</v>
+      </c>
+      <c r="T3" t="s">
+        <v>29</v>
+      </c>
+      <c r="U3" t="s">
+        <v>30</v>
+      </c>
+      <c r="V3" t="s">
+        <v>31</v>
+      </c>
+      <c r="W3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
         <v>23</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C4" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4">
+        <v>750</v>
+      </c>
+      <c r="G4">
+        <v>759</v>
+      </c>
+      <c r="H4">
+        <v>60</v>
+      </c>
+      <c r="I4">
+        <v>40</v>
+      </c>
+      <c r="J4">
+        <v>659</v>
+      </c>
+      <c r="K4">
+        <v>70</v>
+      </c>
+      <c r="L4">
+        <v>110</v>
+      </c>
+      <c r="M4">
+        <v>20</v>
+      </c>
+      <c r="N4">
+        <v>20</v>
+      </c>
+      <c r="O4">
+        <v>749</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>26</v>
+      </c>
+      <c r="R4" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" t="s">
+        <v>28</v>
+      </c>
+      <c r="T4" t="s">
+        <v>29</v>
+      </c>
+      <c r="U4" t="s">
+        <v>30</v>
+      </c>
+      <c r="V4" t="s">
+        <v>31</v>
+      </c>
+      <c r="W4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="E3" t="s">
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5">
+        <v>950</v>
+      </c>
+      <c r="G5">
+        <v>899</v>
+      </c>
+      <c r="H5">
+        <v>90</v>
+      </c>
+      <c r="I5">
+        <v>60</v>
+      </c>
+      <c r="J5">
+        <v>749</v>
+      </c>
+      <c r="K5">
+        <v>90</v>
+      </c>
+      <c r="L5">
+        <v>130</v>
+      </c>
+      <c r="M5">
+        <v>20</v>
+      </c>
+      <c r="N5">
+        <v>20</v>
+      </c>
+      <c r="O5">
+        <v>1039</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="s">
         <v>26</v>
       </c>
-      <c r="F3" t="s">
+      <c r="R5" t="s">
+        <v>36</v>
+      </c>
+      <c r="S5" t="s">
+        <v>37</v>
+      </c>
+      <c r="T5" t="s">
+        <v>38</v>
+      </c>
+      <c r="U5" t="s">
+        <v>39</v>
+      </c>
+      <c r="V5" t="s">
+        <v>40</v>
+      </c>
+      <c r="W5" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
         <v>23</v>
       </c>
-      <c r="G3" t="s">
+      <c r="C6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>41</v>
+      </c>
+      <c r="F6">
+        <v>955</v>
+      </c>
+      <c r="G6">
+        <v>649</v>
+      </c>
+      <c r="H6">
+        <v>50</v>
+      </c>
+      <c r="I6">
+        <v>40</v>
+      </c>
+      <c r="J6">
+        <v>559</v>
+      </c>
+      <c r="K6">
+        <v>60</v>
+      </c>
+      <c r="L6">
+        <v>120</v>
+      </c>
+      <c r="M6">
+        <v>30</v>
+      </c>
+      <c r="N6">
+        <v>30</v>
+      </c>
+      <c r="O6">
+        <v>1039</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>26</v>
+      </c>
+      <c r="R6" t="s">
+        <v>36</v>
+      </c>
+      <c r="S6" t="s">
+        <v>37</v>
+      </c>
+      <c r="T6" t="s">
+        <v>38</v>
+      </c>
+      <c r="U6" t="s">
+        <v>39</v>
+      </c>
+      <c r="V6" t="s">
+        <v>40</v>
+      </c>
+      <c r="W6" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>48</v>
+      </c>
+      <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="H3" t="s">
+      <c r="C7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7">
+        <v>850</v>
+      </c>
+      <c r="G7">
+        <v>749</v>
+      </c>
+      <c r="H7">
+        <v>70</v>
+      </c>
+      <c r="I7">
+        <v>50</v>
+      </c>
+      <c r="J7">
+        <v>629</v>
+      </c>
+      <c r="K7">
+        <v>80</v>
+      </c>
+      <c r="L7">
+        <v>140</v>
+      </c>
+      <c r="M7">
+        <v>30</v>
+      </c>
+      <c r="N7">
+        <v>30</v>
+      </c>
+      <c r="O7">
+        <v>1039</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>26</v>
+      </c>
+      <c r="R7" t="s">
+        <v>36</v>
+      </c>
+      <c r="S7" t="s">
+        <v>37</v>
+      </c>
+      <c r="T7" t="s">
+        <v>38</v>
+      </c>
+      <c r="U7" t="s">
+        <v>39</v>
+      </c>
+      <c r="V7" t="s">
+        <v>40</v>
+      </c>
+      <c r="W7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8">
+        <v>750</v>
+      </c>
+      <c r="G8">
+        <v>699</v>
+      </c>
+      <c r="H8">
+        <v>60</v>
+      </c>
+      <c r="I8">
+        <v>40</v>
+      </c>
+      <c r="J8">
+        <v>599</v>
+      </c>
+      <c r="K8">
+        <v>70</v>
+      </c>
+      <c r="L8">
+        <v>110</v>
+      </c>
+      <c r="M8">
+        <v>20</v>
+      </c>
+      <c r="N8">
+        <v>20</v>
+      </c>
+      <c r="O8">
+        <v>1039</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>26</v>
+      </c>
+      <c r="R8" t="s">
+        <v>36</v>
+      </c>
+      <c r="S8" t="s">
+        <v>37</v>
+      </c>
+      <c r="T8" t="s">
+        <v>38</v>
+      </c>
+      <c r="U8" t="s">
+        <v>39</v>
+      </c>
+      <c r="V8" t="s">
+        <v>40</v>
+      </c>
+      <c r="W8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="s">
         <v>23</v>
       </c>
-      <c r="J3" t="s">
+      <c r="C9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9">
+        <v>950</v>
+      </c>
+      <c r="G9">
+        <v>799</v>
+      </c>
+      <c r="H9">
+        <v>80</v>
+      </c>
+      <c r="I9">
+        <v>50</v>
+      </c>
+      <c r="J9">
+        <v>669</v>
+      </c>
+      <c r="K9">
+        <v>70</v>
+      </c>
+      <c r="L9">
+        <v>110</v>
+      </c>
+      <c r="M9">
+        <v>20</v>
+      </c>
+      <c r="N9">
+        <v>20</v>
+      </c>
+      <c r="O9">
+        <v>1388</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>26</v>
+      </c>
+      <c r="R9" t="s">
+        <v>42</v>
+      </c>
+      <c r="S9" t="s">
+        <v>43</v>
+      </c>
+      <c r="T9" t="s">
+        <v>29</v>
+      </c>
+      <c r="U9" t="s">
+        <v>44</v>
+      </c>
+      <c r="V9" t="s">
+        <v>45</v>
+      </c>
+      <c r="W9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" t="s">
         <v>23</v>
       </c>
-      <c r="K3" t="s">
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10">
+        <v>955</v>
+      </c>
+      <c r="G10">
+        <v>849</v>
+      </c>
+      <c r="H10">
+        <v>90</v>
+      </c>
+      <c r="I10">
+        <v>60</v>
+      </c>
+      <c r="J10">
+        <v>699</v>
+      </c>
+      <c r="K10">
+        <v>80</v>
+      </c>
+      <c r="L10">
+        <v>120</v>
+      </c>
+      <c r="M10">
+        <v>20</v>
+      </c>
+      <c r="N10">
+        <v>20</v>
+      </c>
+      <c r="O10">
+        <v>1388</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>26</v>
+      </c>
+      <c r="R10" t="s">
+        <v>42</v>
+      </c>
+      <c r="S10" t="s">
+        <v>43</v>
+      </c>
+      <c r="T10" t="s">
+        <v>29</v>
+      </c>
+      <c r="U10" t="s">
+        <v>44</v>
+      </c>
+      <c r="V10" t="s">
+        <v>45</v>
+      </c>
+      <c r="W10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" t="s">
         <v>23</v>
       </c>
-      <c r="L3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M3" t="s">
-        <v>23</v>
-      </c>
-      <c r="N3" t="s">
-        <v>23</v>
-      </c>
-      <c r="O3" t="s">
-        <v>23</v>
-      </c>
-      <c r="P3" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>23</v>
-      </c>
-      <c r="R3" t="s">
-        <v>23</v>
-      </c>
-      <c r="S3" t="s">
-        <v>23</v>
-      </c>
-      <c r="T3" t="s">
-        <v>23</v>
-      </c>
-      <c r="U3" t="s">
-        <v>23</v>
-      </c>
-      <c r="V3" t="s">
-        <v>23</v>
-      </c>
-      <c r="W3" t="s">
-        <v>23</v>
+      <c r="C11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11">
+        <v>700</v>
+      </c>
+      <c r="G11">
+        <v>699</v>
+      </c>
+      <c r="H11">
+        <v>60</v>
+      </c>
+      <c r="I11">
+        <v>40</v>
+      </c>
+      <c r="J11">
+        <v>599</v>
+      </c>
+      <c r="K11">
+        <v>70</v>
+      </c>
+      <c r="L11">
+        <v>100</v>
+      </c>
+      <c r="M11">
+        <v>20</v>
+      </c>
+      <c r="N11">
+        <v>20</v>
+      </c>
+      <c r="O11">
+        <v>1388</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>26</v>
+      </c>
+      <c r="R11" t="s">
+        <v>42</v>
+      </c>
+      <c r="S11" t="s">
+        <v>43</v>
+      </c>
+      <c r="T11" t="s">
+        <v>29</v>
+      </c>
+      <c r="U11" t="s">
+        <v>44</v>
+      </c>
+      <c r="V11" t="s">
+        <v>45</v>
+      </c>
+      <c r="W11" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>